<commit_message>
chore: backup catalog data
</commit_message>
<xml_diff>
--- a/data/xpoint-products.xlsx
+++ b/data/xpoint-products.xlsx
@@ -67,66 +67,69 @@
     <t>نام محصول</t>
   </si>
   <si>
+    <t>برند</t>
+  </si>
+  <si>
+    <t>کد محصول</t>
+  </si>
+  <si>
     <t>راهنما</t>
   </si>
   <si>
+    <t>قیمت نقد</t>
+  </si>
+  <si>
     <t>نمایش محصول</t>
   </si>
   <si>
-    <t>برند</t>
+    <t>دسته‌بندی</t>
+  </si>
+  <si>
+    <t>توضیحات</t>
   </si>
   <si>
     <t>فقط محصولی در سایت نمایش داده می‌شود که نام، برند، کد محصول و قیمت نقد داشته باشد.</t>
   </si>
   <si>
-    <t>کد محصول</t>
-  </si>
-  <si>
     <t>موجود کردن</t>
   </si>
   <si>
+    <t>عکس</t>
+  </si>
+  <si>
     <t>قیمت نقد را وارد کنید؛ ردیف به رنگ سبز درمی‌آید و محصول در سایت موجود محسوب می‌شود.</t>
   </si>
   <si>
-    <t>قیمت نقد</t>
+    <t>دسته‌بندی اصلی</t>
   </si>
   <si>
     <t>ناموجود کردن</t>
   </si>
   <si>
+    <t>گروه اصلی</t>
+  </si>
+  <si>
     <t>فقط قیمت نقد را خالی کنید؛ محصول از سایت حذف می‌شود ولی اطلاعات آن در شیت باقی می‌ماند.</t>
   </si>
   <si>
     <t>فهرست برندها</t>
   </si>
   <si>
-    <t>دسته‌بندی</t>
-  </si>
-  <si>
     <t>برند تمام ردیف‌های معتبر در فیلتر سایت باقی می‌ماند؛ حتی اگر قیمت محصول خالی باشد.</t>
   </si>
   <si>
+    <t>iPhone 17 Pro Max 512GB ZA/A Non Active Silver</t>
+  </si>
+  <si>
     <t>عکس محصول</t>
   </si>
   <si>
-    <t>توضیحات</t>
-  </si>
-  <si>
     <t>لینک عمومی فایل Google Drive یا شناسه فایل عکس را در ستون «عکس» قرار دهید.</t>
   </si>
   <si>
-    <t>عکس</t>
-  </si>
-  <si>
-    <t>دسته‌بندی اصلی</t>
-  </si>
-  <si>
     <t>متن ستون «توضیحات» در پنجره جزئیات محصول نمایش داده می‌شود.</t>
   </si>
   <si>
-    <t>گروه اصلی</t>
-  </si>
-  <si>
     <t>آرایشی و بهداشتی</t>
   </si>
   <si>
@@ -136,9 +139,6 @@
     <t>دسته‌بندی‌های مجاز</t>
   </si>
   <si>
-    <t>iPhone 17 Pro Max 512GB ZA/A Non Active Silver</t>
-  </si>
-  <si>
     <t>یخچال، ظرفشویی، لباسشویی، موبایل، لپ تاپ، اکسسوری، گجت، اسپیکر، تبلت، کنسول بازی، شارژر، تلویزیون، گجت خانگی</t>
   </si>
   <si>
@@ -148,13 +148,13 @@
     <t>Product</t>
   </si>
   <si>
+    <t>پوشه بنرها</t>
+  </si>
+  <si>
+    <t>baner</t>
+  </si>
+  <si>
     <t>اپل</t>
-  </si>
-  <si>
-    <t>پوشه بنرها</t>
-  </si>
-  <si>
-    <t>baner</t>
   </si>
   <si>
     <t>1109410629</t>
@@ -7758,16 +7758,16 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -8044,40 +8044,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>21</v>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>32</v>
@@ -8102,7 +8102,7 @@
         <v>35</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C3" s="7" t="s">
         <v>36</v>
@@ -8129,7 +8129,7 @@
         <v>38</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>39</v>
@@ -8154,7 +8154,7 @@
         <v>41</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>42</v>
@@ -8177,7 +8177,7 @@
         <v>43</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>44</v>
@@ -8204,7 +8204,7 @@
         <v>47</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>48</v>
@@ -8231,7 +8231,7 @@
         <v>49</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>50</v>
@@ -8258,7 +8258,7 @@
         <v>51</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>52</v>
@@ -8285,7 +8285,7 @@
         <v>53</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>54</v>
@@ -8312,7 +8312,7 @@
         <v>55</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>56</v>
@@ -8337,7 +8337,7 @@
         <v>57</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>58</v>
@@ -8360,7 +8360,7 @@
         <v>59</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>60</v>
@@ -8385,7 +8385,7 @@
         <v>61</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>62</v>
@@ -8408,7 +8408,7 @@
         <v>63</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>64</v>
@@ -8431,7 +8431,7 @@
         <v>65</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>66</v>
@@ -8456,7 +8456,7 @@
         <v>67</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>68</v>
@@ -8479,7 +8479,7 @@
         <v>69</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>70</v>
@@ -8504,7 +8504,7 @@
         <v>71</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>72</v>
@@ -8527,7 +8527,7 @@
         <v>73</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>74</v>
@@ -8550,7 +8550,7 @@
         <v>75</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>76</v>
@@ -8573,7 +8573,7 @@
         <v>77</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>78</v>
@@ -8596,7 +8596,7 @@
         <v>79</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>80</v>
@@ -8619,7 +8619,7 @@
         <v>81</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>82</v>
@@ -8642,7 +8642,7 @@
         <v>83</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>84</v>
@@ -8665,7 +8665,7 @@
         <v>85</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>86</v>
@@ -8688,7 +8688,7 @@
         <v>87</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>88</v>
@@ -8711,7 +8711,7 @@
         <v>89</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>90</v>
@@ -8734,7 +8734,7 @@
         <v>91</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>92</v>
@@ -8757,7 +8757,7 @@
         <v>93</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>94</v>
@@ -8780,7 +8780,7 @@
         <v>95</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>96</v>
@@ -8803,7 +8803,7 @@
         <v>97</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>98</v>
@@ -8826,7 +8826,7 @@
         <v>99</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C33" s="7" t="s">
         <v>100</v>
@@ -8849,7 +8849,7 @@
         <v>101</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>102</v>
@@ -8872,7 +8872,7 @@
         <v>103</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>104</v>
@@ -8895,7 +8895,7 @@
         <v>105</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C36" s="7" t="s">
         <v>106</v>
@@ -8918,7 +8918,7 @@
         <v>107</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C37" s="7" t="s">
         <v>108</v>
@@ -8941,7 +8941,7 @@
         <v>109</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C38" s="7" t="s">
         <v>110</v>
@@ -8964,7 +8964,7 @@
         <v>111</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C39" s="7" t="s">
         <v>112</v>
@@ -8987,7 +8987,7 @@
         <v>113</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C40" s="7" t="s">
         <v>114</v>
@@ -9010,7 +9010,7 @@
         <v>115</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>116</v>
@@ -9033,7 +9033,7 @@
         <v>117</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C42" s="7" t="s">
         <v>118</v>
@@ -9056,7 +9056,7 @@
         <v>119</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C43" s="7" t="s">
         <v>120</v>
@@ -9079,7 +9079,7 @@
         <v>121</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C44" s="7" t="s">
         <v>122</v>
@@ -9102,7 +9102,7 @@
         <v>123</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C45" s="7" t="s">
         <v>124</v>
@@ -9125,7 +9125,7 @@
         <v>125</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>126</v>
@@ -9148,7 +9148,7 @@
         <v>127</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C47" s="7" t="s">
         <v>128</v>
@@ -9171,7 +9171,7 @@
         <v>129</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C48" s="7" t="s">
         <v>130</v>
@@ -9194,7 +9194,7 @@
         <v>131</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C49" s="7" t="s">
         <v>132</v>
@@ -9217,7 +9217,7 @@
         <v>133</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C50" s="7" t="s">
         <v>134</v>
@@ -9240,7 +9240,7 @@
         <v>135</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C51" s="7" t="s">
         <v>136</v>
@@ -9263,7 +9263,7 @@
         <v>137</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C52" s="7" t="s">
         <v>138</v>
@@ -9286,7 +9286,7 @@
         <v>139</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C53" s="7" t="s">
         <v>140</v>
@@ -9309,7 +9309,7 @@
         <v>141</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C54" s="7" t="s">
         <v>142</v>
@@ -9332,7 +9332,7 @@
         <v>143</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C55" s="7" t="s">
         <v>144</v>
@@ -9355,7 +9355,7 @@
         <v>145</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C56" s="7" t="s">
         <v>146</v>
@@ -9378,7 +9378,7 @@
         <v>147</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>148</v>
@@ -9403,7 +9403,7 @@
         <v>149</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>150</v>
@@ -9428,7 +9428,7 @@
         <v>151</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C59" s="7" t="s">
         <v>152</v>
@@ -9453,7 +9453,7 @@
         <v>153</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C60" s="7" t="s">
         <v>154</v>
@@ -9478,7 +9478,7 @@
         <v>155</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C61" s="7" t="s">
         <v>156</v>
@@ -9503,7 +9503,7 @@
         <v>157</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C62" s="7" t="s">
         <v>158</v>
@@ -9528,7 +9528,7 @@
         <v>159</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C63" s="7" t="s">
         <v>160</v>
@@ -9553,7 +9553,7 @@
         <v>161</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C64" s="7" t="s">
         <v>162</v>
@@ -9578,7 +9578,7 @@
         <v>163</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C65" s="7" t="s">
         <v>164</v>
@@ -9603,7 +9603,7 @@
         <v>165</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C66" s="7" t="s">
         <v>166</v>
@@ -9626,7 +9626,7 @@
         <v>169</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C67" s="7" t="s">
         <v>170</v>
@@ -9649,7 +9649,7 @@
         <v>171</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C68" s="7" t="s">
         <v>172</v>
@@ -9674,7 +9674,7 @@
         <v>174</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>175</v>
@@ -9699,7 +9699,7 @@
         <v>174</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C70" s="7" t="s">
         <v>178</v>
@@ -9724,7 +9724,7 @@
         <v>179</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C71" s="7" t="s">
         <v>180</v>
@@ -9749,7 +9749,7 @@
         <v>182</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C72" s="7" t="s">
         <v>183</v>
@@ -9772,7 +9772,7 @@
         <v>184</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C73" s="7" t="s">
         <v>185</v>
@@ -9797,7 +9797,7 @@
         <v>174</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C74" s="7" t="s">
         <v>186</v>
@@ -9822,7 +9822,7 @@
         <v>187</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C75" s="7" t="s">
         <v>188</v>
@@ -9847,7 +9847,7 @@
         <v>189</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C76" s="7" t="s">
         <v>190</v>
@@ -18839,9 +18839,7 @@
       <c r="C463" s="7" t="s">
         <v>984</v>
       </c>
-      <c r="D463" s="11">
-        <v>3389000.0</v>
-      </c>
+      <c r="D463" s="11"/>
       <c r="E463" s="6" t="s">
         <v>33</v>
       </c>
@@ -18868,9 +18866,7 @@
       <c r="C464" s="7" t="s">
         <v>987</v>
       </c>
-      <c r="D464" s="11">
-        <v>3163000.0</v>
-      </c>
+      <c r="D464" s="11"/>
       <c r="E464" s="6" t="s">
         <v>33</v>
       </c>
@@ -18897,9 +18893,7 @@
       <c r="C465" s="7" t="s">
         <v>990</v>
       </c>
-      <c r="D465" s="11">
-        <v>7853000.0</v>
-      </c>
+      <c r="D465" s="11"/>
       <c r="E465" s="6" t="s">
         <v>33</v>
       </c>
@@ -18926,9 +18920,7 @@
       <c r="C466" s="7" t="s">
         <v>992</v>
       </c>
-      <c r="D466" s="11">
-        <v>4327000.0</v>
-      </c>
+      <c r="D466" s="11"/>
       <c r="E466" s="6" t="s">
         <v>33</v>
       </c>
@@ -24181,9 +24173,7 @@
       <c r="C693" s="7" t="s">
         <v>1488</v>
       </c>
-      <c r="D693" s="11">
-        <v>3613000.0</v>
-      </c>
+      <c r="D693" s="11"/>
       <c r="E693" s="6" t="s">
         <v>33</v>
       </c>
@@ -24210,9 +24200,7 @@
       <c r="C694" s="7" t="s">
         <v>1492</v>
       </c>
-      <c r="D694" s="11">
-        <v>3613000.0</v>
-      </c>
+      <c r="D694" s="11"/>
       <c r="E694" s="6" t="s">
         <v>33</v>
       </c>
@@ -24408,9 +24396,7 @@
       <c r="C702" s="7" t="s">
         <v>1509</v>
       </c>
-      <c r="D702" s="11">
-        <v>5921000.0</v>
-      </c>
+      <c r="D702" s="11"/>
       <c r="E702" s="6" t="s">
         <v>33</v>
       </c>
@@ -24437,9 +24423,7 @@
       <c r="C703" s="7" t="s">
         <v>1512</v>
       </c>
-      <c r="D703" s="11">
-        <v>4406000.0</v>
-      </c>
+      <c r="D703" s="11"/>
       <c r="E703" s="6" t="s">
         <v>33</v>
       </c>
@@ -24466,9 +24450,7 @@
       <c r="C704" s="7" t="s">
         <v>1515</v>
       </c>
-      <c r="D704" s="11">
-        <v>3898000.0</v>
-      </c>
+      <c r="D704" s="11"/>
       <c r="E704" s="6" t="s">
         <v>33</v>
       </c>
@@ -24659,14 +24641,12 @@
         <v>1532</v>
       </c>
       <c r="B712" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C712" s="7" t="s">
         <v>1533</v>
       </c>
-      <c r="D712" s="11">
-        <v>4.52E7</v>
-      </c>
+      <c r="D712" s="11"/>
       <c r="E712" s="6" t="s">
         <v>167</v>
       </c>
@@ -24688,14 +24668,12 @@
         <v>1536</v>
       </c>
       <c r="B713" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C713" s="7" t="s">
         <v>1537</v>
       </c>
-      <c r="D713" s="11">
-        <v>3.729E7</v>
-      </c>
+      <c r="D713" s="11"/>
       <c r="E713" s="6" t="s">
         <v>167</v>
       </c>
@@ -24717,14 +24695,12 @@
         <v>1538</v>
       </c>
       <c r="B714" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C714" s="7" t="s">
         <v>1539</v>
       </c>
-      <c r="D714" s="11">
-        <v>2.5538E7</v>
-      </c>
+      <c r="D714" s="11"/>
       <c r="E714" s="6" t="s">
         <v>167</v>
       </c>
@@ -24746,7 +24722,7 @@
         <v>1540</v>
       </c>
       <c r="B715" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C715" s="7" t="s">
         <v>1541</v>
@@ -24769,7 +24745,7 @@
         <v>1542</v>
       </c>
       <c r="B716" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C716" s="7" t="s">
         <v>1543</v>
@@ -24792,7 +24768,7 @@
         <v>1544</v>
       </c>
       <c r="B717" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C717" s="7" t="s">
         <v>1545</v>
@@ -24815,7 +24791,7 @@
         <v>1546</v>
       </c>
       <c r="B718" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C718" s="7" t="s">
         <v>1547</v>
@@ -24840,7 +24816,7 @@
         <v>1548</v>
       </c>
       <c r="B719" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C719" s="7" t="s">
         <v>1549</v>
@@ -24865,7 +24841,7 @@
         <v>1550</v>
       </c>
       <c r="B720" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C720" s="7" t="s">
         <v>1551</v>
@@ -24890,7 +24866,7 @@
         <v>1552</v>
       </c>
       <c r="B721" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C721" s="7" t="s">
         <v>1553</v>
@@ -24913,7 +24889,7 @@
         <v>1554</v>
       </c>
       <c r="B722" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C722" s="7" t="s">
         <v>1555</v>
@@ -24936,7 +24912,7 @@
         <v>1556</v>
       </c>
       <c r="B723" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C723" s="7" t="s">
         <v>1557</v>
@@ -24959,7 +24935,7 @@
         <v>1558</v>
       </c>
       <c r="B724" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C724" s="7" t="s">
         <v>1559</v>
@@ -24982,7 +24958,7 @@
         <v>1560</v>
       </c>
       <c r="B725" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C725" s="7" t="s">
         <v>1561</v>
@@ -25005,7 +24981,7 @@
         <v>1562</v>
       </c>
       <c r="B726" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C726" s="7" t="s">
         <v>1563</v>
@@ -25028,7 +25004,7 @@
         <v>1564</v>
       </c>
       <c r="B727" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C727" s="7" t="s">
         <v>1565</v>
@@ -25051,7 +25027,7 @@
         <v>1566</v>
       </c>
       <c r="B728" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C728" s="7" t="s">
         <v>1567</v>
@@ -25074,7 +25050,7 @@
         <v>1568</v>
       </c>
       <c r="B729" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C729" s="7" t="s">
         <v>1569</v>
@@ -25097,7 +25073,7 @@
         <v>1570</v>
       </c>
       <c r="B730" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C730" s="7" t="s">
         <v>1571</v>
@@ -25120,7 +25096,7 @@
         <v>1572</v>
       </c>
       <c r="B731" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C731" s="7" t="s">
         <v>1573</v>
@@ -25147,14 +25123,12 @@
         <v>1574</v>
       </c>
       <c r="B732" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C732" s="7" t="s">
         <v>1575</v>
       </c>
-      <c r="D732" s="11">
-        <v>3108000.0</v>
-      </c>
+      <c r="D732" s="11"/>
       <c r="E732" s="6" t="s">
         <v>632</v>
       </c>
@@ -25176,7 +25150,7 @@
         <v>1578</v>
       </c>
       <c r="B733" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C733" s="7" t="s">
         <v>1579</v>
@@ -25201,7 +25175,7 @@
         <v>1580</v>
       </c>
       <c r="B734" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C734" s="7" t="s">
         <v>1581</v>
@@ -25224,7 +25198,7 @@
         <v>1582</v>
       </c>
       <c r="B735" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C735" s="7" t="s">
         <v>1583</v>
@@ -25249,7 +25223,7 @@
         <v>1584</v>
       </c>
       <c r="B736" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C736" s="7" t="s">
         <v>1585</v>
@@ -25272,7 +25246,7 @@
         <v>1586</v>
       </c>
       <c r="B737" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C737" s="7" t="s">
         <v>1587</v>
@@ -25295,7 +25269,7 @@
         <v>1588</v>
       </c>
       <c r="B738" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C738" s="7" t="s">
         <v>1589</v>
@@ -25318,7 +25292,7 @@
         <v>1590</v>
       </c>
       <c r="B739" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C739" s="7" t="s">
         <v>1591</v>
@@ -25343,7 +25317,7 @@
         <v>1592</v>
       </c>
       <c r="B740" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C740" s="7" t="s">
         <v>1593</v>
@@ -25368,7 +25342,7 @@
         <v>1594</v>
       </c>
       <c r="B741" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C741" s="7" t="s">
         <v>1595</v>
@@ -25393,7 +25367,7 @@
         <v>1596</v>
       </c>
       <c r="B742" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C742" s="7" t="s">
         <v>1597</v>
@@ -25418,7 +25392,7 @@
         <v>1598</v>
       </c>
       <c r="B743" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C743" s="7" t="s">
         <v>1599</v>
@@ -25443,7 +25417,7 @@
         <v>1600</v>
       </c>
       <c r="B744" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C744" s="7" t="s">
         <v>1601</v>
@@ -25611,9 +25585,7 @@
       <c r="C751" s="7" t="s">
         <v>1619</v>
       </c>
-      <c r="D751" s="11">
-        <v>2498000.0</v>
-      </c>
+      <c r="D751" s="11"/>
       <c r="E751" s="6" t="s">
         <v>167</v>
       </c>
@@ -26001,9 +25973,7 @@
       <c r="C767" s="7" t="s">
         <v>1653</v>
       </c>
-      <c r="D767" s="11">
-        <v>7.4579E7</v>
-      </c>
+      <c r="D767" s="11"/>
       <c r="E767" s="6" t="s">
         <v>33</v>
       </c>
@@ -26026,9 +25996,7 @@
       <c r="C768" s="7" t="s">
         <v>1655</v>
       </c>
-      <c r="D768" s="11">
-        <v>7.4579E7</v>
-      </c>
+      <c r="D768" s="11"/>
       <c r="E768" s="6" t="s">
         <v>33</v>
       </c>
@@ -26074,9 +26042,7 @@
       <c r="C770" s="7" t="s">
         <v>1659</v>
       </c>
-      <c r="D770" s="11">
-        <v>1.25429E8</v>
-      </c>
+      <c r="D770" s="11"/>
       <c r="E770" s="6" t="s">
         <v>33</v>
       </c>
@@ -26101,9 +26067,7 @@
       <c r="C771" s="7" t="s">
         <v>1662</v>
       </c>
-      <c r="D771" s="11">
-        <v>1.25429E8</v>
-      </c>
+      <c r="D771" s="11"/>
       <c r="E771" s="6" t="s">
         <v>33</v>
       </c>
@@ -26128,9 +26092,7 @@
       <c r="C772" s="7" t="s">
         <v>1664</v>
       </c>
-      <c r="D772" s="11">
-        <v>1.25429E8</v>
-      </c>
+      <c r="D772" s="11"/>
       <c r="E772" s="6" t="s">
         <v>33</v>
       </c>
@@ -26155,9 +26117,7 @@
       <c r="C773" s="7" t="s">
         <v>1666</v>
       </c>
-      <c r="D773" s="11">
-        <v>1.25429E8</v>
-      </c>
+      <c r="D773" s="11"/>
       <c r="E773" s="6" t="s">
         <v>33</v>
       </c>
@@ -26182,9 +26142,7 @@
       <c r="C774" s="7" t="s">
         <v>1668</v>
       </c>
-      <c r="D774" s="11">
-        <v>1.57069E8</v>
-      </c>
+      <c r="D774" s="11"/>
       <c r="E774" s="6" t="s">
         <v>33</v>
       </c>
@@ -26263,9 +26221,7 @@
       <c r="C777" s="7" t="s">
         <v>1677</v>
       </c>
-      <c r="D777" s="11">
-        <v>1.1865E7</v>
-      </c>
+      <c r="D777" s="11"/>
       <c r="E777" s="6" t="s">
         <v>632</v>
       </c>
@@ -26319,9 +26275,7 @@
       <c r="C779" s="7" t="s">
         <v>1685</v>
       </c>
-      <c r="D779" s="11">
-        <v>8927000.0</v>
-      </c>
+      <c r="D779" s="11"/>
       <c r="E779" s="6" t="s">
         <v>632</v>
       </c>
@@ -26394,9 +26348,7 @@
       <c r="C782" s="7" t="s">
         <v>1694</v>
       </c>
-      <c r="D782" s="11">
-        <v>1.1865E8</v>
-      </c>
+      <c r="D782" s="11"/>
       <c r="E782" s="6" t="s">
         <v>1347</v>
       </c>
@@ -26448,9 +26400,7 @@
       <c r="C784" s="7" t="s">
         <v>1701</v>
       </c>
-      <c r="D784" s="11">
-        <v>8.8705E7</v>
-      </c>
+      <c r="D784" s="11"/>
       <c r="E784" s="6" t="s">
         <v>1347</v>
       </c>
@@ -26477,9 +26427,7 @@
       <c r="C785" s="7" t="s">
         <v>1703</v>
       </c>
-      <c r="D785" s="11">
-        <v>6.328E7</v>
-      </c>
+      <c r="D785" s="11"/>
       <c r="E785" s="6" t="s">
         <v>1347</v>
       </c>
@@ -27271,9 +27219,7 @@
       <c r="C819" s="7" t="s">
         <v>1778</v>
       </c>
-      <c r="D819" s="11">
-        <v>1.85319E8</v>
-      </c>
+      <c r="D819" s="11"/>
       <c r="E819" s="6" t="s">
         <v>33</v>
       </c>
@@ -28479,9 +28425,7 @@
       <c r="C869" s="7" t="s">
         <v>1863</v>
       </c>
-      <c r="D869" s="11">
-        <v>6.1019E7</v>
-      </c>
+      <c r="D869" s="11"/>
       <c r="E869" s="6" t="s">
         <v>33</v>
       </c>
@@ -28748,9 +28692,7 @@
       <c r="C880" s="7" t="s">
         <v>1885</v>
       </c>
-      <c r="D880" s="11">
-        <v>1.33339E8</v>
-      </c>
+      <c r="D880" s="11"/>
       <c r="E880" s="6" t="s">
         <v>33</v>
       </c>
@@ -29046,9 +28988,7 @@
       <c r="C892" s="7" t="s">
         <v>1909</v>
       </c>
-      <c r="D892" s="11">
-        <v>1.7289E8</v>
-      </c>
+      <c r="D892" s="11"/>
       <c r="E892" s="6" t="s">
         <v>1339</v>
       </c>
@@ -29075,9 +29015,7 @@
       <c r="C893" s="7" t="s">
         <v>1913</v>
       </c>
-      <c r="D893" s="11">
-        <v>1.4803E7</v>
-      </c>
+      <c r="D893" s="11"/>
       <c r="E893" s="6" t="s">
         <v>1339</v>
       </c>
@@ -29104,9 +29042,7 @@
       <c r="C894" s="7" t="s">
         <v>1918</v>
       </c>
-      <c r="D894" s="11">
-        <v>9368000.0</v>
-      </c>
+      <c r="D894" s="11"/>
       <c r="E894" s="6" t="s">
         <v>1339</v>
       </c>
@@ -29179,9 +29115,7 @@
       <c r="C897" s="7" t="s">
         <v>1927</v>
       </c>
-      <c r="D897" s="11">
-        <v>1.4916E7</v>
-      </c>
+      <c r="D897" s="11"/>
       <c r="E897" s="6" t="s">
         <v>1339</v>
       </c>
@@ -30050,9 +29984,7 @@
       <c r="C934" s="7" t="s">
         <v>1995</v>
       </c>
-      <c r="D934" s="11">
-        <v>8927000.0</v>
-      </c>
+      <c r="D934" s="11"/>
       <c r="E934" s="6" t="s">
         <v>1608</v>
       </c>
@@ -30612,9 +30544,7 @@
       <c r="C958" s="7" t="s">
         <v>2059</v>
       </c>
-      <c r="D958" s="11">
-        <v>3955000.0</v>
-      </c>
+      <c r="D958" s="11"/>
       <c r="E958" s="6" t="s">
         <v>632</v>
       </c>
@@ -31241,9 +31171,7 @@
       <c r="C985" s="7" t="s">
         <v>2122</v>
       </c>
-      <c r="D985" s="11">
-        <v>5.4579E7</v>
-      </c>
+      <c r="D985" s="11"/>
       <c r="E985" s="6" t="s">
         <v>1608</v>
       </c>
@@ -31270,9 +31198,7 @@
       <c r="C986" s="7" t="s">
         <v>2126</v>
       </c>
-      <c r="D986" s="11">
-        <v>4.0567E7</v>
-      </c>
+      <c r="D986" s="11"/>
       <c r="E986" s="6" t="s">
         <v>1608</v>
       </c>
@@ -31322,9 +31248,7 @@
       <c r="C988" s="7" t="s">
         <v>2131</v>
       </c>
-      <c r="D988" s="11">
-        <v>9492000.0</v>
-      </c>
+      <c r="D988" s="11"/>
       <c r="E988" s="6" t="s">
         <v>632</v>
       </c>
@@ -31405,9 +31329,7 @@
       <c r="C991" s="7" t="s">
         <v>2143</v>
       </c>
-      <c r="D991" s="11">
-        <v>6554000.0</v>
-      </c>
+      <c r="D991" s="11"/>
       <c r="E991" s="6" t="s">
         <v>632</v>
       </c>
@@ -31484,9 +31406,7 @@
       <c r="C994" s="7" t="s">
         <v>2150</v>
       </c>
-      <c r="D994" s="11">
-        <v>8475000.0</v>
-      </c>
+      <c r="D994" s="11"/>
       <c r="E994" s="6" t="s">
         <v>1608</v>
       </c>
@@ -31561,9 +31481,7 @@
       <c r="C997" s="7" t="s">
         <v>2157</v>
       </c>
-      <c r="D997" s="11">
-        <v>7.797E7</v>
-      </c>
+      <c r="D997" s="11"/>
       <c r="E997" s="6" t="s">
         <v>1608</v>
       </c>
@@ -31636,9 +31554,7 @@
       <c r="C1000" s="7" t="s">
         <v>2165</v>
       </c>
-      <c r="D1000" s="11">
-        <v>8.7009E7</v>
-      </c>
+      <c r="D1000" s="11"/>
       <c r="E1000" s="6" t="s">
         <v>1347</v>
       </c>
@@ -31807,9 +31723,7 @@
       <c r="C1007" s="7" t="s">
         <v>2185</v>
       </c>
-      <c r="D1007" s="11">
-        <v>4.2939E7</v>
-      </c>
+      <c r="D1007" s="11"/>
       <c r="E1007" s="6" t="s">
         <v>167</v>
       </c>
@@ -31836,9 +31750,7 @@
       <c r="C1008" s="7" t="s">
         <v>2189</v>
       </c>
-      <c r="D1008" s="11">
-        <v>6102000.0</v>
-      </c>
+      <c r="D1008" s="11"/>
       <c r="E1008" s="6" t="s">
         <v>167</v>
       </c>
@@ -31936,9 +31848,7 @@
       <c r="C1012" s="7" t="s">
         <v>2199</v>
       </c>
-      <c r="D1012" s="11">
-        <v>3615000.0</v>
-      </c>
+      <c r="D1012" s="11"/>
       <c r="E1012" s="6" t="s">
         <v>33</v>
       </c>
@@ -31965,9 +31875,7 @@
       <c r="C1013" s="7" t="s">
         <v>2201</v>
       </c>
-      <c r="D1013" s="11">
-        <v>4745000.0</v>
-      </c>
+      <c r="D1013" s="11"/>
       <c r="E1013" s="6" t="s">
         <v>33</v>
       </c>
@@ -31994,9 +31902,7 @@
       <c r="C1014" s="7" t="s">
         <v>2203</v>
       </c>
-      <c r="D1014" s="11">
-        <v>8135000.0</v>
-      </c>
+      <c r="D1014" s="11"/>
       <c r="E1014" s="6" t="s">
         <v>33</v>
       </c>
@@ -32069,9 +31975,7 @@
       <c r="C1017" s="7" t="s">
         <v>2209</v>
       </c>
-      <c r="D1017" s="11">
-        <v>3.0509E7</v>
-      </c>
+      <c r="D1017" s="11"/>
       <c r="E1017" s="6" t="s">
         <v>33</v>
       </c>
@@ -32098,9 +32002,7 @@
       <c r="C1018" s="7" t="s">
         <v>2212</v>
       </c>
-      <c r="D1018" s="11">
-        <v>3.0509E7</v>
-      </c>
+      <c r="D1018" s="11"/>
       <c r="E1018" s="6" t="s">
         <v>33</v>
       </c>
@@ -32127,9 +32029,7 @@
       <c r="C1019" s="7" t="s">
         <v>2214</v>
       </c>
-      <c r="D1019" s="11">
-        <v>3.0509E7</v>
-      </c>
+      <c r="D1019" s="11"/>
       <c r="E1019" s="6" t="s">
         <v>33</v>
       </c>
@@ -32156,9 +32056,7 @@
       <c r="C1020" s="7" t="s">
         <v>2216</v>
       </c>
-      <c r="D1020" s="11">
-        <v>6.2149E7</v>
-      </c>
+      <c r="D1020" s="11"/>
       <c r="E1020" s="6" t="s">
         <v>33</v>
       </c>
@@ -32185,9 +32083,7 @@
       <c r="C1021" s="7" t="s">
         <v>2220</v>
       </c>
-      <c r="D1021" s="11">
-        <v>6.2149E7</v>
-      </c>
+      <c r="D1021" s="11"/>
       <c r="E1021" s="6" t="s">
         <v>33</v>
       </c>
@@ -32241,9 +32137,7 @@
       <c r="C1023" s="7" t="s">
         <v>2224</v>
       </c>
-      <c r="D1023" s="11">
-        <v>7.1189E7</v>
-      </c>
+      <c r="D1023" s="11"/>
       <c r="E1023" s="6" t="s">
         <v>33</v>
       </c>
@@ -32270,9 +32164,7 @@
       <c r="C1024" s="7" t="s">
         <v>2227</v>
       </c>
-      <c r="D1024" s="11">
-        <v>7.1189E7</v>
-      </c>
+      <c r="D1024" s="11"/>
       <c r="E1024" s="6" t="s">
         <v>33</v>
       </c>
@@ -32299,9 +32191,7 @@
       <c r="C1025" s="7" t="s">
         <v>2229</v>
       </c>
-      <c r="D1025" s="11">
-        <v>7.1189E7</v>
-      </c>
+      <c r="D1025" s="11"/>
       <c r="E1025" s="6" t="s">
         <v>33</v>
       </c>
@@ -32328,9 +32218,7 @@
       <c r="C1026" s="7" t="s">
         <v>2231</v>
       </c>
-      <c r="D1026" s="11">
-        <v>8.5879E7</v>
-      </c>
+      <c r="D1026" s="11"/>
       <c r="E1026" s="6" t="s">
         <v>33</v>
       </c>
@@ -32357,9 +32245,7 @@
       <c r="C1027" s="7" t="s">
         <v>2235</v>
       </c>
-      <c r="D1027" s="11">
-        <v>8.5879E7</v>
-      </c>
+      <c r="D1027" s="11"/>
       <c r="E1027" s="6" t="s">
         <v>33</v>
       </c>
@@ -32386,9 +32272,7 @@
       <c r="C1028" s="7" t="s">
         <v>2237</v>
       </c>
-      <c r="D1028" s="11">
-        <v>8.5879E7</v>
-      </c>
+      <c r="D1028" s="11"/>
       <c r="E1028" s="6" t="s">
         <v>33</v>
       </c>
@@ -32415,9 +32299,7 @@
       <c r="C1029" s="7" t="s">
         <v>2239</v>
       </c>
-      <c r="D1029" s="11">
-        <v>8.8817E7</v>
-      </c>
+      <c r="D1029" s="11"/>
       <c r="E1029" s="6" t="s">
         <v>33</v>
       </c>
@@ -32442,9 +32324,7 @@
       <c r="C1030" s="7" t="s">
         <v>2241</v>
       </c>
-      <c r="D1030" s="11">
-        <v>8.8817E7</v>
-      </c>
+      <c r="D1030" s="11"/>
       <c r="E1030" s="6" t="s">
         <v>33</v>
       </c>
@@ -32498,9 +32378,7 @@
       <c r="C1032" s="7" t="s">
         <v>2248</v>
       </c>
-      <c r="D1032" s="11">
-        <v>1.70629E8</v>
-      </c>
+      <c r="D1032" s="11"/>
       <c r="E1032" s="6" t="s">
         <v>33</v>
       </c>
@@ -32552,9 +32430,7 @@
       <c r="C1034" s="7" t="s">
         <v>2252</v>
       </c>
-      <c r="D1034" s="11">
-        <v>1.77409E8</v>
-      </c>
+      <c r="D1034" s="11"/>
       <c r="E1034" s="6" t="s">
         <v>33</v>
       </c>
@@ -32581,9 +32457,7 @@
       <c r="C1035" s="7" t="s">
         <v>2255</v>
       </c>
-      <c r="D1035" s="11">
-        <v>1.77409E8</v>
-      </c>
+      <c r="D1035" s="11"/>
       <c r="E1035" s="6" t="s">
         <v>33</v>
       </c>
@@ -32610,9 +32484,7 @@
       <c r="C1036" s="7" t="s">
         <v>2257</v>
       </c>
-      <c r="D1036" s="11">
-        <v>1.77409E8</v>
-      </c>
+      <c r="D1036" s="11"/>
       <c r="E1036" s="6" t="s">
         <v>33</v>
       </c>
@@ -32639,9 +32511,7 @@
       <c r="C1037" s="7" t="s">
         <v>2259</v>
       </c>
-      <c r="D1037" s="11">
-        <v>9.7179E7</v>
-      </c>
+      <c r="D1037" s="11"/>
       <c r="E1037" s="6" t="s">
         <v>33</v>
       </c>
@@ -32668,9 +32538,7 @@
       <c r="C1038" s="7" t="s">
         <v>2263</v>
       </c>
-      <c r="D1038" s="11">
-        <v>9.7179E7</v>
-      </c>
+      <c r="D1038" s="11"/>
       <c r="E1038" s="6" t="s">
         <v>33</v>
       </c>
@@ -32724,9 +32592,7 @@
       <c r="C1040" s="7" t="s">
         <v>2268</v>
       </c>
-      <c r="D1040" s="11">
-        <v>9.9439E7</v>
-      </c>
+      <c r="D1040" s="11"/>
       <c r="E1040" s="6" t="s">
         <v>33</v>
       </c>
@@ -32753,9 +32619,7 @@
       <c r="C1041" s="7" t="s">
         <v>2270</v>
       </c>
-      <c r="D1041" s="11">
-        <v>9.9439E7</v>
-      </c>
+      <c r="D1041" s="11"/>
       <c r="E1041" s="6" t="s">
         <v>33</v>
       </c>
@@ -33378,7 +33242,7 @@
         <v>2321</v>
       </c>
       <c r="B1067" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1067" s="7" t="s">
         <v>2322</v>
@@ -33756,7 +33620,7 @@
         <v>2353</v>
       </c>
       <c r="B1083" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C1083" s="7" t="s">
         <v>2354</v>
@@ -34065,9 +33929,7 @@
       <c r="C1095" s="7" t="s">
         <v>2385</v>
       </c>
-      <c r="D1095" s="11">
-        <v>1.15104E8</v>
-      </c>
+      <c r="D1095" s="11"/>
       <c r="E1095" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34175,9 +34037,7 @@
       <c r="C1099" s="7" t="s">
         <v>2398</v>
       </c>
-      <c r="D1099" s="11">
-        <v>1.451516E8</v>
-      </c>
+      <c r="D1099" s="11"/>
       <c r="E1099" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34231,9 +34091,7 @@
       <c r="C1101" s="7" t="s">
         <v>2406</v>
       </c>
-      <c r="D1101" s="11">
-        <v>1.013727E8</v>
-      </c>
+      <c r="D1101" s="11"/>
       <c r="E1101" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34260,9 +34118,7 @@
       <c r="C1102" s="7" t="s">
         <v>2409</v>
       </c>
-      <c r="D1102" s="11">
-        <v>6.456681E7</v>
-      </c>
+      <c r="D1102" s="11"/>
       <c r="E1102" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34289,9 +34145,7 @@
       <c r="C1103" s="7" t="s">
         <v>2412</v>
       </c>
-      <c r="D1103" s="11">
-        <v>2.5696E7</v>
-      </c>
+      <c r="D1103" s="11"/>
       <c r="E1103" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34318,9 +34172,7 @@
       <c r="C1104" s="7" t="s">
         <v>2417</v>
       </c>
-      <c r="D1104" s="11">
-        <v>2.56344E7</v>
-      </c>
+      <c r="D1104" s="11"/>
       <c r="E1104" s="6" t="s">
         <v>1608</v>
       </c>
@@ -34347,9 +34199,7 @@
       <c r="C1105" s="7" t="s">
         <v>2421</v>
       </c>
-      <c r="D1105" s="11">
-        <v>2.53506E7</v>
-      </c>
+      <c r="D1105" s="11"/>
       <c r="E1105" s="6" t="s">
         <v>1608</v>
       </c>
@@ -39527,91 +39377,91 @@
   </cols>
   <sheetData>
     <row r="1" ht="33.0" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" ht="33.0" customHeight="1">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
+      <c r="A2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" ht="33.0" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" ht="33.0" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" ht="33.0" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" ht="33.0" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" ht="33.0" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" ht="33.0" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" ht="33.0" customHeight="1">
-      <c r="A5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" ht="33.0" customHeight="1">
-      <c r="A6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" ht="33.0" customHeight="1">
-      <c r="A7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>20</v>
+      <c r="B7" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="8" ht="33.0" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>23</v>
       </c>
+      <c r="B8" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="9" ht="33.0" customHeight="1">
-      <c r="A9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="3" t="s">
+      <c r="A9" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="10" ht="33.0" customHeight="1">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" ht="33.0" customHeight="1">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>